<commit_message>
docs: outreach cadence + weekly funnel sheet in prospecting workbook
</commit_message>
<xml_diff>
--- a/docs/pitch/prospeccao-musa.xlsx
+++ b/docs/pitch/prospeccao-musa.xlsx
@@ -11,16 +11,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incubadoras" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundos" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Museus" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funil semanal" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1" calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +63,12 @@
       <color rgb="001F2937"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Inter"/>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -86,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -98,6 +107,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -696,7 +708,7 @@
       <c r="I2" s="6" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -754,7 +766,7 @@
       <c r="I3" s="6" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -812,7 +824,7 @@
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -870,7 +882,7 @@
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -928,7 +940,7 @@
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -986,7 +998,7 @@
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -1044,7 +1056,7 @@
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1102,7 +1114,7 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1160,7 +1172,7 @@
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1316,7 +1328,7 @@
       <c r="I2" s="6" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -1374,7 +1386,7 @@
       <c r="I3" s="6" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -1432,7 +1444,7 @@
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -1490,7 +1502,7 @@
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -1548,7 +1560,7 @@
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -1606,7 +1618,7 @@
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -1664,7 +1676,7 @@
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -1722,7 +1734,7 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -1780,7 +1792,7 @@
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1838,7 +1850,7 @@
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -1896,7 +1908,7 @@
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Enviar e-mail frio + one-pager</t>
+          <t>D0: e-mail frio + one-pager → D4: follow-up → D10: LinkedIn</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -2048,7 +2060,7 @@
       <c r="I2" s="6" t="inlineStr"/>
       <c r="J2" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K2" s="6" t="inlineStr">
@@ -2102,7 +2114,7 @@
       <c r="I3" s="6" t="inlineStr"/>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -2156,7 +2168,7 @@
       <c r="I4" s="6" t="inlineStr"/>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
@@ -2210,7 +2222,7 @@
       <c r="I5" s="6" t="inlineStr"/>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
@@ -2264,7 +2276,7 @@
       <c r="I6" s="6" t="inlineStr"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K6" s="6" t="inlineStr">
@@ -2318,7 +2330,7 @@
       <c r="I7" s="6" t="inlineStr"/>
       <c r="J7" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K7" s="6" t="inlineStr">
@@ -2372,7 +2384,7 @@
       <c r="I8" s="6" t="inlineStr"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K8" s="6" t="inlineStr">
@@ -2426,7 +2438,7 @@
       <c r="I9" s="6" t="inlineStr"/>
       <c r="J9" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -2480,7 +2492,7 @@
       <c r="I10" s="6" t="inlineStr"/>
       <c r="J10" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -2534,7 +2546,7 @@
       <c r="I11" s="6" t="inlineStr"/>
       <c r="J11" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K11" s="6" t="inlineStr">
@@ -2588,7 +2600,7 @@
       <c r="I12" s="6" t="inlineStr"/>
       <c r="J12" s="6" t="inlineStr">
         <is>
-          <t>Mapear contato da diretoria</t>
+          <t>D0: e-mail/telefone à diretoria → D7: follow-up → D15: visita ou chamada</t>
         </is>
       </c>
       <c r="K12" s="6" t="inlineStr">
@@ -2613,4 +2625,516 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Funil semanal — acompanhamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>As linhas de status contam AO VIVO das abas Incubadoras/Fundos/Museus. Para congelar o histórico: ao fechar a semana, copie a linha e Cole especial → Valores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Semana de</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Não contatado</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Contatado</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Respondeu</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Reunião marcada</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Proposta enviada</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Fechado</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Descartado</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Total em cadastro</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>Observações</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I6" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I7" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J7" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="7" t="n"/>
+      <c r="C8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I8" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J8" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I9" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J9" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I10" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J10" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="n"/>
+      <c r="C11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I11" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J11" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="n"/>
+      <c r="C12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I12" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J12" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="n"/>
+      <c r="C13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I13" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J13" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I14" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J14" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="7" t="n"/>
+      <c r="C15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I15" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J15" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I16" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J16" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,C$5)+COUNTIF(Fundos!$H$2:$H$100,C$5)+COUNTIF(Museus!$H$2:$H$100,C$5)</f>
+        <v/>
+      </c>
+      <c r="D17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,D$5)+COUNTIF(Fundos!$H$2:$H$100,D$5)+COUNTIF(Museus!$H$2:$H$100,D$5)</f>
+        <v/>
+      </c>
+      <c r="E17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,E$5)+COUNTIF(Fundos!$H$2:$H$100,E$5)+COUNTIF(Museus!$H$2:$H$100,E$5)</f>
+        <v/>
+      </c>
+      <c r="F17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,F$5)+COUNTIF(Fundos!$H$2:$H$100,F$5)+COUNTIF(Museus!$H$2:$H$100,F$5)</f>
+        <v/>
+      </c>
+      <c r="G17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,G$5)+COUNTIF(Fundos!$H$2:$H$100,G$5)+COUNTIF(Museus!$H$2:$H$100,G$5)</f>
+        <v/>
+      </c>
+      <c r="H17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,H$5)+COUNTIF(Fundos!$H$2:$H$100,H$5)+COUNTIF(Museus!$H$2:$H$100,H$5)</f>
+        <v/>
+      </c>
+      <c r="I17" s="8">
+        <f>COUNTIF(Incubadoras!$H$2:$H$100,I$5)+COUNTIF(Fundos!$H$2:$H$100,I$5)+COUNTIF(Museus!$H$2:$H$100,I$5)</f>
+        <v/>
+      </c>
+      <c r="J17" s="9">
+        <f>COUNTA(Incubadoras!$A$2:$A$100)+COUNTA(Fundos!$A$2:$A$100)+COUNTA(Museus!$A$2:$A$100)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>